<commit_message>
feat: enhance personal goal tracking with completion details and approval history
- Added new fields to PersonalGoalListDto for completion evidence, certification URL, and summary.
- Updated GoalSetEvaluationInfoDto to include approval history.
- Expanded GoalDto with additional properties for goal tracking and activity management.
- Modified dashboard to reflect updated performance metrics (high performers threshold changed to ≥85%).
- Refactored role checks in DashboardComponent and HeaderComponent for better role management.
- Introduced new SubmitTlCombinedReviewDto for combined review submissions.
- Updated evaluation service to handle new review submission logic.
- Removed outdated dev-cache script and improved docker management script for better development workflow.
- Created migration to add new columns for personal goal completion details in the database.
- Documented new development workflow in RUN_PROJECT_DOCKER_DEV.md.
</commit_message>
<xml_diff>
--- a/docs/test-data/empovate360-import-users-v2.xlsx
+++ b/docs/test-data/empovate360-import-users-v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>gm.ceo@empovate.test</t>
@@ -628,7 +627,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>superman.admin@empovate.test</t>
@@ -696,7 +694,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -764,7 +761,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>hod.engineering@empovate.test</t>
@@ -832,7 +828,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -900,7 +895,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -968,7 +962,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>gm.ceo@empovate.test</t>
@@ -1036,7 +1029,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>superman.admin@empovate.test</t>
@@ -1104,7 +1096,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -1172,7 +1163,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -1240,7 +1230,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>admin.ops@empovate.test</t>
@@ -1308,7 +1297,6 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
@@ -1376,13 +1364,146 @@
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>rm.platform@empovate.test</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
+        <is>
+          <t>tl.platform@empovate.test</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>employee.three@empovate.test</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Employee Three</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>rm.platform@empovate.test</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ENG-PLT</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Platform Engineering</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>rm.platform@empovate.test</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>tl.platform@empovate.test</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>employee.four@empovate.test</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Employee Four</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>rm.platform@empovate.test</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ENG-PLT</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Platform Engineering</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>rm.platform@empovate.test</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>tl.platform@empovate.test</t>
         </is>

</xml_diff>